<commit_message>
changed name of Evo-M1-Traits-Data-restricted to Evo-M1-Trait-Data-restricted
</commit_message>
<xml_diff>
--- a/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
+++ b/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
@@ -872,13 +872,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4BD65FE-23F1-4124-AF0C-16FC855C9322}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3540A9F9-0193-496F-ADC6-41E6D7E475E1}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCE9C34D-25D7-4627-8A36-38899DEA22E5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9209FDD8-0D98-4A09-BE24-FCB968EA0E20}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{52205C13-F0DE-4081-9000-448C736B0740}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1683CEA4-EA34-4BE8-806E-F88C8565886F}"/>
 </file>
</xml_diff>

<commit_message>
cleaning dead files and fixing broken scripts
</commit_message>
<xml_diff>
--- a/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
+++ b/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
@@ -872,13 +872,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3540A9F9-0193-496F-ADC6-41E6D7E475E1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A58D9FF-CDD6-40E8-BC7E-E3177DE18D98}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9209FDD8-0D98-4A09-BE24-FCB968EA0E20}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9EFE32A9-240F-4667-8B78-13CA4D39C4D3}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1683CEA4-EA34-4BE8-806E-F88C8565886F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3B008DD0-3384-446E-A46D-054571F50EA2}"/>
 </file>
</xml_diff>

<commit_message>
Refresh Shiny app data 2026-08-24 10:07
</commit_message>
<xml_diff>
--- a/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
+++ b/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
@@ -872,13 +872,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A58D9FF-CDD6-40E8-BC7E-E3177DE18D98}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1182AB1C-F0F1-47E9-A46B-FF5D453BBC44}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9EFE32A9-240F-4667-8B78-13CA4D39C4D3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CFFE946F-277E-43C4-8365-76998D0D9FAC}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3B008DD0-3384-446E-A46D-054571F50EA2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AA82B8A-05A9-43C2-A02D-EC0BB50E48DF}"/>
 </file>
</xml_diff>

<commit_message>
Refresh Shiny app data 2026-09-05 06:53
</commit_message>
<xml_diff>
--- a/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
+++ b/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
@@ -872,13 +872,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E25C8C5-CC47-408D-82DB-E22E558EE892}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7BCE8B23-D43E-4EFB-83F2-B7F53E6A7463}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{373A22E8-3B37-4B51-80B9-AA226C2A357E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{741B4450-C174-4A79-AD48-47166C63F340}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{422AF71D-CA0E-448D-8DEA-5D02527431E5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{68D71E6D-2971-4EFB-8B9E-2F1AF1723998}"/>
 </file>
</xml_diff>